<commit_message>
Add re-review sheet after BA rewrite of AMP-2548
Round-2 scoring of the rewritten story (AC1-AC10 + IA1-IA4): 5 of 6 CPO
requirements covered, R5 partial; references ACP-230/265/266/268 verified.
Ten open issues logged, three P1 (Staff ID orphaning, unmatched code
handling, round-robin scope contradiction).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YVZU6rcGxvxzfBwFWwCyhr
</commit_message>
<xml_diff>
--- a/output/02-reporting-hierarchy/20260903-002-reporting-hierarchy-cpo-gap.xlsx
+++ b/output/02-reporting-hierarchy/20260903-002-reporting-hierarchy-cpo-gap.xlsx
@@ -7,9 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Gap Analysis" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Staff ID vs UTM" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="ADIB Reference" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Re-review 03-09 PM" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Gap Analysis" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Staff ID vs UTM" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="ADIB Reference" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -107,7 +108,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -129,11 +130,44 @@
         <color rgb="FFD9D9D9"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFD9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFD9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFD9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -181,6 +215,10 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -546,6 +584,622 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="56" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Re-review — After BA Rewrite (03/09/2026 PM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>AMP-2548 rewritten to AC1–AC10 + IA1–IA4 per feedback · new refs ACP-230/265/266/268 verified valid · mockup + BRD attached</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Coverage now: 5 Covered · 1 Partially covered · 0 Not covered — but 3 P1 design defects found in the new ACs (see Open Issues below). Round-1 baseline kept on sheet 'Gap Analysis'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="4" customHeight="1">
+      <c r="A4" s="4" t="n"/>
+      <c r="B4" s="4" t="n"/>
+      <c r="C4" s="4" t="n"/>
+      <c r="D4" s="4" t="n"/>
+      <c r="E4" s="4" t="n"/>
+      <c r="F4" s="4" t="n"/>
+    </row>
+    <row r="6" ht="26" customHeight="1">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Ref</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Requirement</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Now covered by</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>What remains</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="84" customHeight="1">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>Staff sees own applications only</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>AC1 Staff ID field (unique, IEM001, maps to salesagentCode) · AC4 case attribution (UTM / QR-manual / round-robin) · AC5 own-only pre-filter · AC10 maker/checker</t>
+        </is>
+      </c>
+      <c r="D7" s="21" t="inlineStr">
+        <is>
+          <t>Covered</t>
+        </is>
+      </c>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>Design defect open: Staff ID is editable (AC1/AC10) while attribution is immutable and matched at query time (AC4/AC5) — changing a Staff ID orphans the user's application history. See Issue 1.</t>
+        </is>
+      </c>
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="84" customHeight="1">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>Manager sees team applications</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="inlineStr">
+        <is>
+          <t>AC6 unlimited-depth subtree + own cases, Context aligned · AC8 lifecycle rules (cycle IEM002, deactivation guard IEM003, real-time RM change)</t>
+        </is>
+      </c>
+      <c r="D8" s="21" t="inlineStr">
+        <is>
+          <t>Covered</t>
+        </is>
+      </c>
+      <c r="E8" s="14" t="inlineStr">
+        <is>
+          <t>Depth contradiction resolved; lifecycle covered for managers. Staff-level offboarding (deactivating a tagged, non-manager user) still undefined — Issue 5.</t>
+        </is>
+      </c>
+      <c r="F8" s="14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="84" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>Case tagging basis — Staff ID or UTM</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>Context + AC4 adopt Staff ID as the tag; UTM is the carrier (salesagentCode) per recommendation · IA4 documents the AMP-3323 link</t>
+        </is>
+      </c>
+      <c r="D9" s="21" t="inlineStr">
+        <is>
+          <t>Covered</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>Decision adopted as recommended. Precedence between capture channels ('evaluated in order' vs ADIB's 'latest successful wins') needs one rule — Issue 4. Unmatched/stale codes undefined — Issue 2.</t>
+        </is>
+      </c>
+      <c r="F9" s="11" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="84" customHeight="1">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>Ops / admin retain full visibility</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="inlineStr">
+        <is>
+          <t>AC7 'View All Applications' permission — role-level, default off, includes untagged apps, migration note</t>
+        </is>
+      </c>
+      <c r="D10" s="21" t="inlineStr">
+        <is>
+          <t>Covered</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="inlineStr">
+        <is>
+          <t>Open decision parked in IA4: same permission as AMP-3323 'View All Application Sources' or separate — confirm with Channel team, assign owner. Role list at migration still to be defined.</t>
+        </is>
+      </c>
+      <c r="F10" s="14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="84" customHeight="1">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>Unassigned &amp; historical cases</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>AC4 untagged rule (View-All only) · IA2 migration options (bulk backfill vs grant View-All at go-live) · round-robin fallback</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>Partially covered</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="inlineStr">
+        <is>
+          <t>Mechanisms written but two decisions not made: (1) migration option a or b; (2) round-robin is listed as an AC4 mechanism yet IA2 says 'may require a separate ticket' — in-scope or dependency must be settled now. Issue 3.</t>
+        </is>
+      </c>
+      <c r="F11" s="11" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="84" customHeight="1">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>R6</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>Report Enquiry follows same visibility</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>AC9 scoping incl. exports · refs corrected to ACP-230 (Report Enquiry, Ready for Core Dev) + ACP-265/266/268 (Report List 1–3, US Approved) — all verified valid 03/09</t>
+        </is>
+      </c>
+      <c r="D12" s="21" t="inlineStr">
+        <is>
+          <t>Covered</t>
+        </is>
+      </c>
+      <c r="E12" s="14" t="inlineStr">
+        <is>
+          <t>References verified. No open item.</t>
+        </is>
+      </c>
+      <c r="F12" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Open Issues — to close before Ready for Dev (P1) / before dev completes (P2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Prio</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>Issue</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>Where</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>Recommendation</t>
+        </is>
+      </c>
+      <c r="F15" s="22" t="n"/>
+    </row>
+    <row r="16" ht="62" customHeight="1">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>Staff ID change orphans application history: AC1/AC10 allow editing Staff ID; AC4 makes attribution immutable; AC5/AC6 match at query time. After a change, apps tagged with the old code match nobody — the staff and their manager lose them, only View-All sees them. AC10's own sample ('Staff ID: — → STF-042') is this exact case.</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>AC1 / AC4 / AC5 / AC10</t>
+        </is>
+      </c>
+      <c r="E16" s="11" t="inlineStr">
+        <is>
+          <t>Store a resolved user reference at origination (recommended — keeps AC8's real-time RM logic consistent), or block Staff ID edits once set and define a re-tag procedure.</t>
+        </is>
+      </c>
+      <c r="F16" s="11" t="n"/>
+    </row>
+    <row r="17" ht="62" customHeight="1">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="inlineStr">
+        <is>
+          <t>Unmatched salesagentCode undefined: a UTM/QR code that matches no active user's Staff ID (typo, leaver, code not yet created) — tagged to nothing? Also no normalization rule (case, trim) for matching.</t>
+        </is>
+      </c>
+      <c r="D17" s="14" t="inlineStr">
+        <is>
+          <t>AC4</t>
+        </is>
+      </c>
+      <c r="E17" s="14" t="inlineStr">
+        <is>
+          <t>Fall through to round-robin (recommended) or explicitly untagged + alert; define case-insensitive exact match.</t>
+        </is>
+      </c>
+      <c r="F17" s="14" t="n"/>
+    </row>
+    <row r="18" ht="62" customHeight="1">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>Round-robin scope contradiction: AC4 mechanism 3 treats round-robin as part of this story; IA2 says it 'may require a separate ticket'. If it slips, every non-UTM/QR case is View-All-only.</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>AC4 / IA2</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="inlineStr">
+        <is>
+          <t>Decide now: write the round-robin ACs into this story (config table per channel/product, ADIB-7172 pattern) or raise the dependency ticket and link it as blocking.</t>
+        </is>
+      </c>
+      <c r="F18" s="11" t="n"/>
+    </row>
+    <row r="19" ht="62" customHeight="1">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C19" s="14" t="inlineStr">
+        <is>
+          <t>Capture precedence: AC4 says mechanisms are 'evaluated in order' (UTM beats QR/manual), but ADIB-5651's production rule is 'latest successful code wins'. Both can occur in one journey (UTM link + staff enters code at branch).</t>
+        </is>
+      </c>
+      <c r="D19" s="14" t="inlineStr">
+        <is>
+          <t>AC4</t>
+        </is>
+      </c>
+      <c r="E19" s="14" t="inlineStr">
+        <is>
+          <t>Pick one rule — recommend latest-successful-wins with every attempt audited (ADIB pattern) — and state it in AC4.</t>
+        </is>
+      </c>
+      <c r="F19" s="14" t="n"/>
+    </row>
+    <row r="20" ht="62" customHeight="1">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>Staff offboarding not covered: AC8 blocks deactivating managers with reports, but says nothing about deactivating a staff user with open tagged applications — who re-assigns their pipeline, and does the manager keep seeing a deactivated user's cases?</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>AC8</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>Add a lifecycle row: block until open cases re-assigned (manual or round-robin), or auto re-assign with audit.</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="n"/>
+    </row>
+    <row r="21" ht="62" customHeight="1">
+      <c r="A21" s="13" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C21" s="14" t="inlineStr">
+        <is>
+          <t>QR/manual capture has no SMBP journey story: ADIB-5651 is another bank's implementation. Which SMBP customer-journey screen captures the code? No baseline referenced.</t>
+        </is>
+      </c>
+      <c r="D21" s="14" t="inlineStr">
+        <is>
+          <t>AC4 mech. 2</t>
+        </is>
+      </c>
+      <c r="E21" s="14" t="inlineStr">
+        <is>
+          <t>Confirm scope with journey team: raise the capture-screen story, or drop mechanism 2 for phase 1 (UTM + round-robin still tag every case).</t>
+        </is>
+      </c>
+      <c r="F21" s="14" t="n"/>
+    </row>
+    <row r="22" ht="62" customHeight="1">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>Tag invisible on screen: AC9 keeps all columns unchanged, so managers cannot see who owns a row and staff cannot see why their list shrank.</t>
+        </is>
+      </c>
+      <c r="D22" s="11" t="inlineStr">
+        <is>
+          <t>AC9</t>
+        </is>
+      </c>
+      <c r="E22" s="11" t="inlineStr">
+        <is>
+          <t>Add 'Assigned To (Sale Staff)' as a Customize Table column (default ON for managers/View-All), show attribution on Application Details + first audit-trail entry (ADIB-7388 / ADIB-6725 precedent).</t>
+        </is>
+      </c>
+      <c r="F22" s="11" t="n"/>
+    </row>
+    <row r="23" ht="62" customHeight="1">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B23" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C23" s="14" t="inlineStr">
+        <is>
+          <t>Two parked decisions without owners: IA2 migration option (bulk backfill vs View-All-for-all at go-live) and IA4 permission unification with AMP-3323.</t>
+        </is>
+      </c>
+      <c r="D23" s="14" t="inlineStr">
+        <is>
+          <t>IA2 / IA4</t>
+        </is>
+      </c>
+      <c r="E23" s="14" t="inlineStr">
+        <is>
+          <t>Assign owner + due date each; migration choice gates the dev estimate, permission choice gates Role Management design.</t>
+        </is>
+      </c>
+      <c r="F23" s="14" t="n"/>
+    </row>
+    <row r="24" ht="62" customHeight="1">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>Nit</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>Uniqueness only validated at Maker save — two pending requests with the same Staff ID both pass, duplicate lands at Checker approval.</t>
+        </is>
+      </c>
+      <c r="D24" s="11" t="inlineStr">
+        <is>
+          <t>AC10</t>
+        </is>
+      </c>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>Re-run uniqueness (and cycle) validation at Checker approval.</t>
+        </is>
+      </c>
+      <c r="F24" s="11" t="n"/>
+    </row>
+    <row r="25" ht="62" customHeight="1">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>Nit</t>
+        </is>
+      </c>
+      <c r="C25" s="14" t="inlineStr">
+        <is>
+          <t>Mockup filename still '03-Level-Reporting-Manager' though the Level concept was removed; message codes IEM001/002/003 not confirmed unused; AC7 assignment wording 'per user, at role or channel level' is ambiguous.</t>
+        </is>
+      </c>
+      <c r="D25" s="14" t="inlineStr">
+        <is>
+          <t>Mockup / AC7</t>
+        </is>
+      </c>
+      <c r="E25" s="14" t="inlineStr">
+        <is>
+          <t>Rename mockup file; confirm codes against the message registry; pin AC7 to the Role Management pattern (ACP-257).</t>
+        </is>
+      </c>
+      <c r="F25" s="14" t="n"/>
+    </row>
+    <row r="27" ht="48" customHeight="1">
+      <c r="A27" s="17" t="inlineStr">
+        <is>
+          <t>VERDICT — Strong rewrite: 5 of 6 CPO requirements now covered, R5 partially; the Staff-ID-vs-UTM recommendation adopted as proposed and all baseline references verified. Not Ready for Dev yet: close Issues 1–3 (P1) first — the Staff ID orphaning defect (Issue 1) breaks R1 over time exactly the way the missing tag did originally.</t>
+        </is>
+      </c>
+      <c r="B27" s="18" t="n"/>
+      <c r="C27" s="18" t="n"/>
+      <c r="D27" s="18" t="n"/>
+      <c r="E27" s="18" t="n"/>
+      <c r="F27" s="18" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="E16:F16"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="E25:F25"/>
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="A27:F27"/>
+    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="E17:F17"/>
+    <mergeCell ref="E18:F18"/>
+    <mergeCell ref="E21:F21"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -893,7 +1547,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1117,9 +1771,6 @@
           <t>RECOMMENDATION — Tag the case with STAFF ID (sale code). Capture it through four channels so every case is tagged: (1) UTM link parameter salesagentCode for digital journeys, (2) QR code scan, (3) manual code input for assisted journeys, (4) round-robin default from a configurable table when nothing is provided — the proven ADIB pattern (ADIB-6725, ADIB-5651, ADIB-7172). Keep UTM for campaign analytics only. The Reporting Manager hierarchy (AMP-2548) then determines who sees whose cases.</t>
         </is>
       </c>
-      <c r="B15" s="18" t="n"/>
-      <c r="C15" s="18" t="n"/>
-      <c r="D15" s="18" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1129,7 +1780,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1437,11 +2088,6 @@
           <t>Suggestion for SMBP: (1) add Sale Code / Staff ID to the Bank Portal user record and tag every application at origination via the four ADIB capture channels; (2) reuse the existing UTM engine as the digital carrier of the staff code instead of building a parallel mechanism; (3) make the default-assignment table configurable per channel with maker/checker, and audit every auto-assignment.</t>
         </is>
       </c>
-      <c r="B15" s="20" t="n"/>
-      <c r="C15" s="20" t="n"/>
-      <c r="D15" s="20" t="n"/>
-      <c r="E15" s="20" t="n"/>
-      <c r="F15" s="20" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>